<commit_message>
Add Customer as secondary actor on Book Ticket use case
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -484,7 +484,7 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -762,7 +762,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Administrator (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Administrator (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Sells a ticket for a chosen show and seat, calculates the price automatically and marks the seat as unavailable.</t>
+          <t>Sells a ticket for a chosen show and seat, calculates the price automatically and marks the seat as unavailable. The customer provides details and receives the ticket.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align actors and database design with real cinema_db schema (Admin/Cashier roles)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Administrator, Cashier</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Administrator, Cashier</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Administrator (primary), Customer (secondary)</t>
+          <t>Cashier (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Administrator (primary), Customer (secondary)</t>
+          <t>Cashier (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Administrator, Cashier</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Authenticates the administrator before granting access to the dashboard.</t>
+          <t>Authenticates the user and opens the dashboard according to the role (ADMIN or CASHIER).</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Application running; a valid admin account exists.</t>
+          <t>Application running; a valid account exists in the users table.</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Administrator authenticated; dashboard opens.</t>
+          <t>User authenticated; dashboard opens with role-based access.</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>1. Enter username and password. 2. System validates against the database. 3. On success, dashboard opens.</t>
+          <t>1. Enter username and password. 2. System validates against the users table and reads the role. 3. On success, dashboard opens (full menu for ADMIN, ticket menu for CASHIER).</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1349,7 +1349,7 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>admin_user</t>
+          <t>users</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -1398,7 +1398,11 @@
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr"/>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>UQ</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -1408,74 +1412,78 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(255)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>movie</t>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('ADMIN','CASHIER')</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>default 'CASHIER'</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Key / Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>movie_id</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>customer_id</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(150)</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr"/>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>genre</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr"/>
@@ -1483,12 +1491,12 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>duration_min</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr"/>
@@ -1496,7 +1504,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>cinema_hall</t>
+          <t>movie</t>
         </is>
       </c>
     </row>
@@ -1520,12 +1528,12 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>hall_id</t>
+          <t>movie_id</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -1537,222 +1545,226 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>hall_name</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr"/>
+          <t>VARCHAR(120)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>UQ</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>seating_capacity</t>
+          <t>genre</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(50)</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr"/>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>movie_show</t>
-        </is>
-      </c>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>cinema_hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Key / Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>show_id</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>movie_id</t>
+          <t>hall_id</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>FK -&gt; movie</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>hall_id</t>
+          <t>hall_name</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(60)</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>FK -&gt; cinema_hall</t>
+          <t>UQ</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>show_date</t>
+          <t>capacity</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>show_time</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr"/>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>movie_show</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>pricing</t>
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Key / Note</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Key / Note</t>
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>pricing_id</t>
+          <t>movie_id</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>FK -&gt; movie</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>day_type</t>
+          <t>hall_id</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10)</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Weekday/Weekend</t>
+          <t>FK -&gt; cinema_hall</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>show_date</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10)</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Adult/Kid</t>
-        </is>
-      </c>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>show_time</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>DECIMAL(8,2)</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr"/>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>UQ(hall_id,date,time)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>ticket</t>
+          <t>pricing_config</t>
         </is>
       </c>
     </row>
@@ -1776,12 +1788,12 @@
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>ticket_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -1793,29 +1805,25 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>show_id</t>
+          <t>weekday_adult</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; movie_show</t>
-        </is>
-      </c>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>seat_number</t>
+          <t>weekday_kid</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10)</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr"/>
@@ -1823,29 +1831,25 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>ticket_type</t>
+          <t>weekend_adult</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10)</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>Adult/Kid</t>
-        </is>
-      </c>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>weekend_kid</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>DECIMAL(8,2)</t>
+          <t>INT(11)</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr"/>
@@ -1853,37 +1857,249 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>customer_name</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="9" t="inlineStr">
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>default CURRENT_TIMESTAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Key / Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>ticket_id</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; movie_show</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>seat_number</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>UQ(show_id,seat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>ticket_type</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Adult','Kid')</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(10,2)</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>purchase_date</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>DATETIME</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr"/>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>default CURRENT_TIMESTAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>show_details</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Key / Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>details_id</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>INT(11)</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>UQ -&gt; movie_show</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>movie_name</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(120)</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>hall_name</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(60)</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A28:C28"/>
+  <mergeCells count="8">
+    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A54:C54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Simplify analysis: clean 2-actor, 16 use case, 6-table cinema design
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -479,12 +479,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -522,7 +522,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Administrator, Cashier</t>
+          <t>Administrator</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Administrator, Cashier</t>
+          <t>Administrator</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Administrator</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Update Cinema Hall</t>
+          <t>View Cinema Halls</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Delete Cinema Hall</t>
+          <t>Add Movie Show</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>View Cinema Halls</t>
+          <t>Update Movie Show</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Add Movie Show</t>
+          <t>Delete Movie Show</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Update Movie Show</t>
+          <t>View / Search Movie Shows</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -697,12 +697,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Delete Movie Show</t>
+          <t>Book Ticket</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Administrator (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -712,12 +712,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>View Movie Shows</t>
+          <t>Cancel Ticket</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Administrator</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Update Ticket Pricing (Weekday/Weekend - Adult/Kid)</t>
+          <t>View Sold Tickets</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -742,117 +742,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>View Ticket Pricing</t>
+          <t>Generate Sales Report</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Book Ticket (Sell Ticket)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Cashier (primary), Customer (secondary)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Select Seat</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Cashier</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Check Seat Availability</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Cashier</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Calculate Ticket Price</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Cashier</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>View Sold Tickets</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Cashier</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Update Ticket</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Cashier</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Cancel / Delete Ticket</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Cashier</t>
+          <t>Administrator</t>
         </is>
       </c>
     </row>
@@ -880,7 +775,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>UC-17  —  Book Ticket (Sell Ticket)</t>
+          <t>UC-13  —  Book Ticket</t>
         </is>
       </c>
       <c r="B1" s="4" t="n"/>
@@ -893,7 +788,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>UC-17</t>
+          <t>UC-13</t>
         </is>
       </c>
     </row>
@@ -905,7 +800,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Book Ticket (Sell Ticket)</t>
+          <t>Book Ticket</t>
         </is>
       </c>
     </row>
@@ -917,7 +812,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Cashier (primary), Customer (secondary)</t>
+          <t>Administrator (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -929,7 +824,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Sells a ticket for a chosen show and seat, calculates the price automatically and marks the seat as unavailable. The customer provides details and receives the ticket.</t>
+          <t>Sells a ticket for a chosen show and seat, records the customer and marks the seat as sold.</t>
         </is>
       </c>
     </row>
@@ -941,7 +836,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Administrator is logged in; a show with a free seat exists; pricing is configured.</t>
+          <t>Administrator is logged in; a show with a free seat exists.</t>
         </is>
       </c>
     </row>
@@ -953,7 +848,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>A ticket record is saved; the chosen seat becomes unavailable.</t>
+          <t>A ticket is saved against the show and customer; the seat becomes unavailable.</t>
         </is>
       </c>
     </row>
@@ -965,7 +860,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>1. Select a movie show. 2. Select a seat (include Select Seat). 3. Check seat is free (include Check Seat Availability). 4. Enter customer details and ticket type (Adult/Kid). 5. System calculates price from pricing rules (include Calculate Ticket Price). 6. Confirm; save ticket and mark seat sold. 7. Show confirmation.</t>
+          <t>1. Select a movie show. 2. Select a seat number. 3. Check seat is free (include Check Seat Availability). 4. Enter customer name and phone. 5. Read show ticket price (include Calculate Ticket Price). 6. Confirm; save ticket and mark seat sold. 7. Show confirmation.</t>
         </is>
       </c>
     </row>
@@ -977,7 +872,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3a. Seat already sold -&gt; ask for another seat. 4a. Invalid/missing input -&gt; validation error, not saved.</t>
+          <t>3a. Seat already sold -&gt; ask for another seat. 4a. Missing details -&gt; validation error, not saved.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +920,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Administrator, Cashier</t>
+          <t>Administrator</t>
         </is>
       </c>
     </row>
@@ -1037,7 +932,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Authenticates the user and opens the dashboard according to the role (ADMIN or CASHIER).</t>
+          <t>Authenticates the administrator before granting access to the system.</t>
         </is>
       </c>
     </row>
@@ -1049,7 +944,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Application running; a valid account exists in the users table.</t>
+          <t>Application running; a valid account exists.</t>
         </is>
       </c>
     </row>
@@ -1061,7 +956,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>User authenticated; dashboard opens with role-based access.</t>
+          <t>Administrator authenticated; main menu opens.</t>
         </is>
       </c>
     </row>
@@ -1073,7 +968,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>1. Enter username and password. 2. System validates against the users table and reads the role. 3. On success, dashboard opens (full menu for ADMIN, ticket menu for CASHIER).</t>
+          <t>1. Enter username and password. 2. System validates against the database. 3. On success, main menu opens.</t>
         </is>
       </c>
     </row>
@@ -1096,7 +991,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UC-15  —  Update Ticket Pricing</t>
+          <t>UC-09  —  Add Movie Show</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -1109,7 +1004,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>UC-15</t>
+          <t>UC-09</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1016,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Update Ticket Pricing</t>
+          <t>Add Movie Show</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1040,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Updates ticket prices that vary by day type (weekday/weekend) and category (adult/kid), without changing code.</t>
+          <t>Schedules a movie in a hall at a given date, time and ticket price.</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1052,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Administrator is logged in.</t>
+          <t>Administrator is logged in; at least one movie and one hall exist.</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1064,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>New prices stored and used automatically by the booking screen.</t>
+          <t>A new show record is stored.</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1076,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>1. Open Pricing Management. 2. System shows current prices. 3. Edit prices and save. 4. Store new prices; bookings use them automatically.</t>
+          <t>1. Open Show Management. 2. Choose movie and hall, enter date, time, ticket price. 3. Click Add. 4. Validate and save, refresh table.</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1088,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>3a. Invalid numeric input -&gt; validation error, prices unchanged.</t>
+          <t>3a. A show already exists for that hall at that date/time -&gt; duplicate error.</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1211,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Replicate this template for the remaining CRUD use cases (Update/Delete/View of Movie, Hall, Show; View Pricing; View/Update/Cancel Ticket; Logout).</t>
+          <t>Replicate this template for: Update/Delete/View Movie, Add/View Hall, Update/Delete/View Show, Cancel Ticket, View Sold Tickets, Generate Sales Report, Logout.</t>
         </is>
       </c>
     </row>
@@ -1338,18 +1233,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>user</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1261,7 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Key / Note</t>
+          <t>Key</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1273,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
+          <t>INT (auto)</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -1398,11 +1293,7 @@
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>UQ</t>
-        </is>
-      </c>
+      <c r="C4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -1417,73 +1308,69 @@
       </c>
       <c r="C5" s="9" t="inlineStr"/>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>ENUM('ADMIN','CASHIER')</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>default 'CASHIER'</t>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>movie</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>customer</t>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Key / Note</t>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>movie_id</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>customer_id</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>VARCHAR(120)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>full_name</t>
+          <t>genre</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>VARCHAR(50)</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr"/>
@@ -1491,12 +1378,12 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr"/>
@@ -1504,7 +1391,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>movie</t>
+          <t>cinema_hall</t>
         </is>
       </c>
     </row>
@@ -1521,19 +1408,19 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Key / Note</t>
+          <t>Key</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>movie_id</t>
+          <t>hall_id</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
+          <t>INT (auto)</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -1545,201 +1432,193 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>hall_name</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(120)</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>UQ</t>
-        </is>
-      </c>
+          <t>VARCHAR(60)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>genre</t>
+          <t>capacity</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr"/>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>duration</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr"/>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>movie_show</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>cinema_hall</t>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Key / Note</t>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>hall_id</t>
+          <t>movie_id</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>FK -&gt; movie</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>hall_name</t>
+          <t>hall_id</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(60)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>UQ</t>
+          <t>FK -&gt; cinema_hall</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>capacity</t>
+          <t>show_date</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>show_time</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr"/>
+    </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>movie_show</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>ticket_price</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Key / Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>show_id</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>movie_id</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; movie</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>hall_id</t>
+          <t>customer_id</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
+          <t>INT (auto)</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>FK -&gt; cinema_hall</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>show_date</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr"/>
@@ -1747,24 +1626,20 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>show_time</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>UQ(hall_id,date,time)</t>
-        </is>
-      </c>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>pricing_config</t>
+          <t>ticket</t>
         </is>
       </c>
     </row>
@@ -1781,19 +1656,19 @@
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Key / Note</t>
+          <t>Key</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>ticket_id</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
+          <t>INT (auto)</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -1805,38 +1680,46 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>weekday_adult</t>
+          <t>show_id</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr"/>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; movie_show</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>weekday_kid</t>
+          <t>customer_id</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr"/>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; customer</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>weekend_adult</t>
+          <t>seat_number</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr"/>
@@ -1844,12 +1727,12 @@
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>weekend_kid</t>
+          <t>price</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>INT(11)</t>
+          <t>DECIMAL(8,2)</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr"/>
@@ -1857,249 +1740,24 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>purchase_date</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>default CURRENT_TIMESTAMP</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>ticket</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Key / Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>ticket_id</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="9" t="inlineStr">
-        <is>
-          <t>show_id</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; movie_show</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>seat_number</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>UQ(show_id,seat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="9" t="inlineStr">
-        <is>
-          <t>customer_id</t>
-        </is>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; customer</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>ticket_type</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>ENUM('Adult','Kid')</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>DECIMAL(10,2)</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>purchase_date</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>default CURRENT_TIMESTAMP</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>show_details</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>Key / Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>details_id</t>
-        </is>
-      </c>
-      <c r="B56" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="9" t="inlineStr">
-        <is>
-          <t>show_id</t>
-        </is>
-      </c>
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>INT(11)</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>UQ -&gt; movie_show</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="inlineStr">
-        <is>
-          <t>movie_name</t>
-        </is>
-      </c>
-      <c r="B58" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(120)</t>
-        </is>
-      </c>
-      <c r="C58" s="9" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="inlineStr">
-        <is>
-          <t>hall_name</t>
-        </is>
-      </c>
-      <c r="B59" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(60)</t>
-        </is>
-      </c>
-      <c r="C59" s="9" t="inlineStr"/>
+          <t>DATETIME</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A44:C44"/>
+  <mergeCells count="6">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A20:C20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Model a realistic cinema system: Customer/Cashier/Manager, 20 use cases, 8 tables
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -479,12 +479,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -517,12 +517,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Register Account</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer</t>
         </is>
       </c>
     </row>
@@ -532,12 +532,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Logout</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier, Manager</t>
         </is>
       </c>
     </row>
@@ -547,12 +547,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Add Movie</t>
+          <t>Logout</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier, Manager</t>
         </is>
       </c>
     </row>
@@ -562,12 +562,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Update Movie</t>
+          <t>Search / Browse Movies</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier</t>
         </is>
       </c>
     </row>
@@ -577,12 +577,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Delete Movie</t>
+          <t>View Showtimes</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier</t>
         </is>
       </c>
     </row>
@@ -592,12 +592,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>View / Search Movies</t>
+          <t>Book Ticket</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier</t>
         </is>
       </c>
     </row>
@@ -607,12 +607,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Add Cinema Hall</t>
+          <t>Select Seats</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier</t>
         </is>
       </c>
     </row>
@@ -622,12 +622,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>View Cinema Halls</t>
+          <t>Make Payment</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Add Movie Show</t>
+          <t>View My Bookings</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Update Movie Show</t>
+          <t>Cancel Booking</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier</t>
         </is>
       </c>
     </row>
@@ -667,12 +667,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Delete Movie Show</t>
+          <t>Validate Ticket at Entrance</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -682,12 +682,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>View / Search Movie Shows</t>
+          <t>Add Movie</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -697,12 +697,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Book Ticket</t>
+          <t>Update Movie</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Administrator (primary), Customer (secondary)</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -712,12 +712,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Cancel Ticket</t>
+          <t>Delete Movie</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -727,12 +727,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>View Sold Tickets</t>
+          <t>Schedule Showtime</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -742,12 +742,72 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Generate Sales Report</t>
+          <t>Update Showtime</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Delete Showtime</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Manage Cinema Halls</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Set Ticket Pricing</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>View Sales Report</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -769,13 +829,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>UC-13  —  Book Ticket</t>
+          <t>UC-06  —  Book Ticket</t>
         </is>
       </c>
       <c r="B1" s="4" t="n"/>
@@ -788,7 +848,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>UC-13</t>
+          <t>UC-06</t>
         </is>
       </c>
     </row>
@@ -812,7 +872,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Administrator (primary), Customer (secondary)</t>
+          <t>Customer (online), Cashier (counter)</t>
         </is>
       </c>
     </row>
@@ -824,7 +884,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Sells a ticket for a chosen show and seat, records the customer and marks the seat as sold.</t>
+          <t>Reserves one or more seats for a showtime, takes payment and issues a ticket.</t>
         </is>
       </c>
     </row>
@@ -836,7 +896,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Administrator is logged in; a show with a free seat exists.</t>
+          <t>Actor is logged in; a showtime with at least one free seat exists.</t>
         </is>
       </c>
     </row>
@@ -848,7 +908,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>A ticket is saved against the show and customer; the seat becomes unavailable.</t>
+          <t>A booking and ticket are saved; the chosen seats are marked sold.</t>
         </is>
       </c>
     </row>
@@ -860,7 +920,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>1. Select a movie show. 2. Select a seat number. 3. Check seat is free (include Check Seat Availability). 4. Enter customer name and phone. 5. Read show ticket price (include Calculate Ticket Price). 6. Confirm; save ticket and mark seat sold. 7. Show confirmation.</t>
+          <t>1. Select a movie and showtime. 2. System shows the seat map. 3. Select seats (include Select Seats). 4. System reserves seats and shows total. 5. Confirm and pay (include Make Payment). 6. On success, save booking, issue ticket(s), mark seats sold. 7. Show ticket with reference.</t>
         </is>
       </c>
     </row>
@@ -872,7 +932,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3a. Seat already sold -&gt; ask for another seat. 4a. Missing details -&gt; validation error, not saved.</t>
+          <t>3a. Seat taken meanwhile -&gt; choose another seat. 5a. Payment fails -&gt; release seats, error, no ticket.</t>
         </is>
       </c>
     </row>
@@ -883,7 +943,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>UC-01  —  Login</t>
+          <t>UC-08  —  Make Payment</t>
         </is>
       </c>
       <c r="B11" s="4" t="n"/>
@@ -896,7 +956,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>UC-01</t>
+          <t>UC-08</t>
         </is>
       </c>
     </row>
@@ -908,7 +968,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Make Payment</t>
         </is>
       </c>
     </row>
@@ -920,7 +980,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Customer, Cashier</t>
         </is>
       </c>
     </row>
@@ -932,7 +992,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Authenticates the administrator before granting access to the system.</t>
+          <t>Charges the customer for a booking.</t>
         </is>
       </c>
     </row>
@@ -944,7 +1004,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Application running; a valid account exists.</t>
+          <t>A booking with a total amount is awaiting payment.</t>
         </is>
       </c>
     </row>
@@ -956,7 +1016,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Administrator authenticated; main menu opens.</t>
+          <t>A payment record is created with status Paid or Failed.</t>
         </is>
       </c>
     </row>
@@ -968,7 +1028,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>1. Enter username and password. 2. System validates against the database. 3. On success, main menu opens.</t>
+          <t>1. Show amount due and methods (Card, Mobile Money, Cash). 2. Choose method, enter details. 3. Process payment, record as Paid.</t>
         </is>
       </c>
     </row>
@@ -980,7 +1040,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2a. Invalid credentials -&gt; show 'Invalid login credentials', stay on login screen.</t>
+          <t>3a. Declined -&gt; record Failed, notify; booking stays unpaid.</t>
         </is>
       </c>
     </row>
@@ -991,7 +1051,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UC-09  —  Add Movie Show</t>
+          <t>UC-15  —  Schedule Showtime</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -1004,7 +1064,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>UC-09</t>
+          <t>UC-15</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1076,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Add Movie Show</t>
+          <t>Schedule Showtime</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1088,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1112,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Administrator is logged in; at least one movie and one hall exist.</t>
+          <t>Manager is logged in; at least one movie and one hall exist.</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1124,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>A new show record is stored.</t>
+          <t>A new showtime is stored.</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1136,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>1. Open Show Management. 2. Choose movie and hall, enter date, time, ticket price. 3. Click Add. 4. Validate and save, refresh table.</t>
+          <t>1. Open Showtime scheduling. 2. Choose movie and hall, enter date, time, ticket price. 3. Save. 4. Validate and store the showtime.</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1148,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>3a. A show already exists for that hall at that date/time -&gt; duplicate error.</t>
+          <t>3a. A showtime already exists for that hall at that date/time -&gt; clash error.</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1159,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>UC-03  —  Add Movie</t>
+          <t>UC-12  —  Add Movie</t>
         </is>
       </c>
       <c r="B31" s="4" t="n"/>
@@ -1112,7 +1172,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>UC-03</t>
+          <t>UC-12</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1196,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Administrator</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1220,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Administrator is logged in.</t>
+          <t>Manager is logged in.</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1244,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>1. Open Movie Management. 2. Enter title, genre, duration. 3. Click Add. 4. Validate and save, refresh table.</t>
+          <t>1. Open Movie Management. 2. Enter title, genre, duration, language, rating. 3. Save. 4. Validate and store the movie.</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1271,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Replicate this template for: Update/Delete/View Movie, Add/View Hall, Update/Delete/View Show, Cancel Ticket, View Sold Tickets, Generate Sales Report, Logout.</t>
+          <t>Replicate this template for: Update/Delete Movie, Update/Delete Showtime, Manage Cinema Halls, Set Ticket Pricing, Register Account, View My Bookings, Cancel Booking, Validate Ticket, View Sales Report, Logout.</t>
         </is>
       </c>
     </row>
@@ -1233,18 +1293,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>user</t>
+          <t>customer</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1328,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>customer_id</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -1285,12 +1345,12 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>username</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr"/>
@@ -1298,466 +1358,740 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
           <t>password</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100)</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>movie</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(255)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>movie_id</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(120)</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>genre</t>
+          <t>staff_id</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr"/>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>duration</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>username</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(50)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr"/>
+    </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>cinema_hall</t>
-        </is>
-      </c>
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>password</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(255)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('MANAGER','CASHIER')</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>movie</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>hall_id</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>movie_id</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>INT (auto)</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>hall_name</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(60)</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>capacity</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>movie_show</t>
-        </is>
-      </c>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(120)</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>genre</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(50)</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>show_id</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>movie_id</t>
+          <t>language</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; movie</t>
-        </is>
-      </c>
+          <t>VARCHAR(40)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>cinema_hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
           <t>hall_id</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>hall_name</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(60)</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>capacity</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>showtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>movie_id</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; movie</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>hall_id</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>FK -&gt; cinema_hall</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>show_date</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>DATE</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>show_time</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>ticket_price</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>DECIMAL(8,2)</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>customer</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>customer_id</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>full_name</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(100)</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>phone</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>ticket</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>ticket_id</t>
+          <t>show_date</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>show_id</t>
+          <t>show_time</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; movie_show</t>
-        </is>
-      </c>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
+          <t>ticket_price</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>FK -&gt; customer</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="9" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; showtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>booking_datetime</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>DATETIME</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Paid','Cancelled','Pending')</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>total_amount</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>ticket_id</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>seat_number</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(8)</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>payment</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>payment_id</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
         <is>
           <t>DECIMAL(8,2)</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="inlineStr">
-        <is>
-          <t>purchase_date</t>
-        </is>
-      </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="C61" s="9" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Card','MobileMoney','Cash')</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>payment_datetime</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="inlineStr">
         <is>
           <t>DATETIME</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr"/>
+      <c r="C63" s="9" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B64" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Paid','Failed')</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="A41:C41"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A26:C26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Model realistic counter-based cinema: Manager/Cashier actors, Customer secondary
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -483,8 +483,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -517,12 +517,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Register Account</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Manager, Cashier</t>
         </is>
       </c>
     </row>
@@ -532,12 +532,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logout</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier, Manager</t>
+          <t>Manager, Cashier</t>
         </is>
       </c>
     </row>
@@ -547,12 +547,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Logout</t>
+          <t>Search / View Movies</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier, Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -562,12 +562,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Search / Browse Movies</t>
+          <t>View Showtimes</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -577,12 +577,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>View Showtimes</t>
+          <t>Sell Ticket</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier</t>
+          <t>Cashier (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -592,12 +592,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Book Ticket</t>
+          <t>Select Seat</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -607,12 +607,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Select Seats</t>
+          <t>Check Seat Availability</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -622,12 +622,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Make Payment</t>
+          <t>Take Payment</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>View My Bookings</t>
+          <t>Cancel Ticket</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Cancel Booking</t>
+          <t>Validate Ticket at Entrance</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Validate Ticket at Entrance</t>
+          <t>View Sold Tickets</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Schedule Showtime</t>
+          <t>Manage Cinema Halls</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Update Showtime</t>
+          <t>Schedule Showtime</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Delete Showtime</t>
+          <t>Update Showtime</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Manage Cinema Halls</t>
+          <t>Delete Showtime</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -835,7 +835,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>UC-06  —  Book Ticket</t>
+          <t>UC-05  —  Sell Ticket</t>
         </is>
       </c>
       <c r="B1" s="4" t="n"/>
@@ -848,7 +848,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>UC-06</t>
+          <t>UC-05</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Book Ticket</t>
+          <t>Sell Ticket</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Customer (online), Cashier (counter)</t>
+          <t>Cashier (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Reserves one or more seats for a showtime, takes payment and issues a ticket.</t>
+          <t>Sells a ticket for a chosen showtime and seat: records the customer, takes payment and marks the seat sold.</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Actor is logged in; a showtime with at least one free seat exists.</t>
+          <t>Cashier is logged in; a showtime with at least one free seat exists.</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>A booking and ticket are saved; the chosen seats are marked sold.</t>
+          <t>A ticket is saved against the showtime and customer; the seat is marked sold.</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>1. Select a movie and showtime. 2. System shows the seat map. 3. Select seats (include Select Seats). 4. System reserves seats and shows total. 5. Confirm and pay (include Make Payment). 6. On success, save booking, issue ticket(s), mark seats sold. 7. Show ticket with reference.</t>
+          <t>1. Select a movie and showtime. 2. Select a seat (include Select Seat). 3. Check seat is free (include Check Seat Availability). 4. Enter customer name, phone and ticket type (Adult/Kid). 5. Show price and take payment (include Take Payment). 6. Save ticket and mark seat sold. 7. Print/show the ticket.</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3a. Seat taken meanwhile -&gt; choose another seat. 5a. Payment fails -&gt; release seats, error, no ticket.</t>
+          <t>3a. Seat already sold -&gt; choose another seat. 5a. Payment not completed -&gt; release seat, no ticket. 4a. Missing details -&gt; validation error.</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>UC-08  —  Make Payment</t>
+          <t>UC-01  —  Login</t>
         </is>
       </c>
       <c r="B11" s="4" t="n"/>
@@ -956,7 +956,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>UC-08</t>
+          <t>UC-01</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Make Payment</t>
+          <t>Login</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Customer, Cashier</t>
+          <t>Manager, Cashier</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Charges the customer for a booking.</t>
+          <t>Authenticates a staff member and opens the menu according to their role.</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>A booking with a total amount is awaiting payment.</t>
+          <t>Application running; a valid staff account exists.</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>A payment record is created with status Paid or Failed.</t>
+          <t>Staff authenticated with role-based access.</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>1. Show amount due and methods (Card, Mobile Money, Cash). 2. Choose method, enter details. 3. Process payment, record as Paid.</t>
+          <t>1. Enter username and password. 2. System validates and reads the role. 3. On success, the menu opens (full for Manager, selling for Cashier).</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>3a. Declined -&gt; record Failed, notify; booking stays unpaid.</t>
+          <t>2a. Invalid credentials -&gt; show 'Invalid login credentials', stay on login screen.</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UC-15  —  Schedule Showtime</t>
+          <t>UC-16  —  Schedule Showtime</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>UC-15</t>
+          <t>UC-16</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>1. Open Movie Management. 2. Enter title, genre, duration, language, rating. 3. Save. 4. Validate and store the movie.</t>
+          <t>1. Open Movie Management. 2. Enter title, genre, duration, rating. 3. Save. 4. Validate and store.</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Replicate this template for: Update/Delete Movie, Update/Delete Showtime, Manage Cinema Halls, Set Ticket Pricing, Register Account, View My Bookings, Cancel Booking, Validate Ticket, View Sales Report, Logout.</t>
+          <t>Replicate this template for: Update/Delete Movie, Manage Cinema Halls, Update/Delete Showtime, Set Ticket Pricing, Search Movies, View Showtimes, Cancel Ticket, Validate Ticket, View Sold Tickets, View Sales Report, Logout.</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1304,7 +1304,7 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>customer</t>
+          <t>staff</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1328,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>customer_id</t>
+          <t>staff_id</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -1358,25 +1358,29 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>username</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr"/>
+          <t>VARCHAR(50)</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>UQ</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>phone</t>
+          <t>password</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr"/>
@@ -1384,12 +1388,12 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>password</t>
+          <t>role</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(255)</t>
+          <t>ENUM('MANAGER','CASHIER')</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr"/>
@@ -1397,7 +1401,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>customer</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1425,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>staff_id</t>
+          <t>customer_id</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -1451,92 +1455,92 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>username</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr"/>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>password</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(255)</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>ENUM('MANAGER','CASHIER')</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr"/>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>movie</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>movie</t>
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>movie_id</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(120)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>movie_id</t>
+          <t>genre</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>VARCHAR(50)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(120)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr"/>
@@ -1544,315 +1548,323 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>genre</t>
+          <t>rating</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr"/>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>duration</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>cinema_hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>hall_id</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>hall_name</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(60)</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>capacity</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>language</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(40)</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>rating</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(10)</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>cinema_hall</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>showtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>movie_id</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; movie</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>hall_id</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>hall_name</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(60)</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>capacity</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>showtime</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; cinema_hall</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>show_id</t>
+          <t>show_date</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>movie_id</t>
+          <t>show_time</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>FK -&gt; movie</t>
+          <t>UQ(hall,date,time)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>hall_id</t>
+          <t>ticket_price</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>ticket_id</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; cinema_hall</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="9" t="inlineStr">
-        <is>
-          <t>show_date</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>DATE</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="9" t="inlineStr">
-        <is>
-          <t>show_time</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="9" t="inlineStr">
-        <is>
-          <t>ticket_price</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>DECIMAL(8,2)</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>booking</t>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; showtime</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; customer</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>booking_id</t>
+          <t>seat_number</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>VARCHAR(8)</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>UQ(show,seat)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>customer_id</t>
+          <t>ticket_type</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; customer</t>
-        </is>
-      </c>
+          <t>ENUM('Adult','Kid')</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>show_id</t>
+          <t>price</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; showtime</t>
-        </is>
-      </c>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>booking_datetime</t>
+          <t>purchase_datetime</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
@@ -1862,236 +1874,14 @@
       </c>
       <c r="C46" s="9" t="inlineStr"/>
     </row>
-    <row r="47">
-      <c r="A47" s="9" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>ENUM('Paid','Cancelled','Pending')</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>total_amount</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>DECIMAL(8,2)</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>ticket</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>ticket_id</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="9" t="inlineStr">
-        <is>
-          <t>booking_id</t>
-        </is>
-      </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; booking</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>seat_number</t>
-        </is>
-      </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(8)</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="9" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="B55" s="9" t="inlineStr">
-        <is>
-          <t>DECIMAL(8,2)</t>
-        </is>
-      </c>
-      <c r="C55" s="9" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>payment</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="inlineStr">
-        <is>
-          <t>payment_id</t>
-        </is>
-      </c>
-      <c r="B59" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C59" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="inlineStr">
-        <is>
-          <t>booking_id</t>
-        </is>
-      </c>
-      <c r="B60" s="9" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C60" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; booking</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="9" t="inlineStr">
-        <is>
-          <t>amount</t>
-        </is>
-      </c>
-      <c r="B61" s="9" t="inlineStr">
-        <is>
-          <t>DECIMAL(8,2)</t>
-        </is>
-      </c>
-      <c r="C61" s="9" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>method</t>
-        </is>
-      </c>
-      <c r="B62" s="9" t="inlineStr">
-        <is>
-          <t>ENUM('Card','MobileMoney','Cash')</t>
-        </is>
-      </c>
-      <c r="C62" s="9" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="9" t="inlineStr">
-        <is>
-          <t>payment_datetime</t>
-        </is>
-      </c>
-      <c r="B63" s="9" t="inlineStr">
-        <is>
-          <t>DATETIME</t>
-        </is>
-      </c>
-      <c r="C63" s="9" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="9" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B64" s="9" t="inlineStr">
-        <is>
-          <t>ENUM('Paid','Failed')</t>
-        </is>
-      </c>
-      <c r="C64" s="9" t="inlineStr"/>
-    </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A41:C41"/>
+  <mergeCells count="6">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mirror lecturer example: full CRUD per entity, 57 use cases, 12 tables
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -110,7 +110,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -479,12 +481,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -517,12 +519,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Add Movie</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Manager, Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -532,12 +534,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Logout</t>
+          <t>Update Movie</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Manager, Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -547,12 +549,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Search / View Movies</t>
+          <t>Delete Movie</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -562,12 +564,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>View Showtimes</t>
+          <t>Search Movie by Title, Genre, Language</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager, Cashier</t>
         </is>
       </c>
     </row>
@@ -577,12 +579,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Sell Ticket</t>
+          <t>Add Genre</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Cashier (primary), Customer (secondary)</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -592,12 +594,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Select Seat</t>
+          <t>Update Genre</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -607,12 +609,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Check Seat Availability</t>
+          <t>Delete Genre</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -622,12 +624,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Take Payment</t>
+          <t>Search Genre by Name</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -637,12 +639,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Cancel Ticket</t>
+          <t>Add Cinema Hall</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -652,12 +654,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Validate Ticket at Entrance</t>
+          <t>Update Cinema Hall</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -667,12 +669,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>View Sold Tickets</t>
+          <t>Delete Cinema Hall</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -682,7 +684,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Add Movie</t>
+          <t>Search Cinema Hall by Name, Type, Capacity</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -697,7 +699,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Update Movie</t>
+          <t>Add Showtime</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -712,7 +714,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Delete Movie</t>
+          <t>Update Showtime</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -727,7 +729,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Manage Cinema Halls</t>
+          <t>Delete Showtime</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -742,12 +744,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Schedule Showtime</t>
+          <t>Search Showtime by Date, Movie, Hall, Time</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Manager, Cashier</t>
         </is>
       </c>
     </row>
@@ -757,12 +759,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Update Showtime</t>
+          <t>Add Customer</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -772,12 +774,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Delete Showtime</t>
+          <t>Update Customer</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -787,7 +789,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Set Ticket Pricing</t>
+          <t>Delete Customer</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -802,12 +804,567 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>View Sales Report</t>
+          <t>Search Customer by Id, Name, Phone</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Add Staff</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Update Staff</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Delete Staff</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Search Staff by Id, Name, Role</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Add Booking</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Cashier, Customer (secondary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Update Booking</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Delete Booking</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Search Booking by Id, Customer, Date, Showtime</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Cashier, Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Add Ticket</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Update Ticket</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Delete Ticket</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Search Ticket by Code, Showtime, Customer</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Cashier, Usher</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Add Payment</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Update Payment</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Delete Payment</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Search Payment by Id, Date, Method, Customer</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Cashier, Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Add Snack</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Update Snack</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Delete Snack</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Search Snack by Name, Category</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Cashier, Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Add Promotion</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Update Promotion</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Delete Promotion</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Search Promotion by Code, Period</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Cashier, Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Post Showtime</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Unpost Showtime</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Select Seat</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Cashier, Customer (secondary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Apply Promotion to Booking</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Generate Ticket</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Validate Ticket at Entrance</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Usher</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Issue Refund</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Cashier, Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Generate Sales Report</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Generate Hall Occupancy Report</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Generate Daily Revenue Report</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Manage User Roles</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Manager, Cashier, Usher</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Manager, Cashier, Usher</t>
         </is>
       </c>
     </row>
@@ -829,13 +1386,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="92" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>UC-05  —  Sell Ticket</t>
+          <t>UC-25  —  Add Booking</t>
         </is>
       </c>
       <c r="B1" s="4" t="n"/>
@@ -848,7 +1405,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>UC-05</t>
+          <t>UC-25</t>
         </is>
       </c>
     </row>
@@ -860,7 +1417,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Sell Ticket</t>
+          <t>Add Booking</t>
         </is>
       </c>
     </row>
@@ -884,7 +1441,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Sells a ticket for a chosen showtime and seat: records the customer, takes payment and marks the seat sold.</t>
+          <t>Creates a booking for a showtime: selects seats, applies any promotion, takes payment and issues the ticket.</t>
         </is>
       </c>
     </row>
@@ -896,7 +1453,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Cashier is logged in; a showtime with at least one free seat exists.</t>
+          <t>Cashier is logged in; a posted showtime with a free seat exists.</t>
         </is>
       </c>
     </row>
@@ -908,7 +1465,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>A ticket is saved against the showtime and customer; the seat is marked sold.</t>
+          <t>A booking, ticket and payment are saved; the seats are marked sold.</t>
         </is>
       </c>
     </row>
@@ -920,7 +1477,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>1. Select a movie and showtime. 2. Select a seat (include Select Seat). 3. Check seat is free (include Check Seat Availability). 4. Enter customer name, phone and ticket type (Adult/Kid). 5. Show price and take payment (include Take Payment). 6. Save ticket and mark seat sold. 7. Print/show the ticket.</t>
+          <t>1. Select a posted showtime. 2. Select seats (include Select Seat). 3. Enter/select the customer. 4. (optional) Apply a promotion (extend Apply Promotion). 5. Show total and take payment (include Add Payment). 6. Save booking and issue ticket (include Generate Ticket); mark seats sold.</t>
         </is>
       </c>
     </row>
@@ -932,7 +1489,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3a. Seat already sold -&gt; choose another seat. 5a. Payment not completed -&gt; release seat, no ticket. 4a. Missing details -&gt; validation error.</t>
+          <t>2a. Seat already sold -&gt; choose another seat. 5a. Payment fails -&gt; release seats, no ticket.</t>
         </is>
       </c>
     </row>
@@ -943,7 +1500,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>UC-01  —  Login</t>
+          <t>UC-50  —  Validate Ticket at Entrance</t>
         </is>
       </c>
       <c r="B11" s="4" t="n"/>
@@ -956,7 +1513,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>UC-01</t>
+          <t>UC-50</t>
         </is>
       </c>
     </row>
@@ -968,7 +1525,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Validate Ticket at Entrance</t>
         </is>
       </c>
     </row>
@@ -980,7 +1537,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Manager, Cashier</t>
+          <t>Usher</t>
         </is>
       </c>
     </row>
@@ -992,7 +1549,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Authenticates a staff member and opens the menu according to their role.</t>
+          <t>Checks a presented ticket is valid for the current showtime and marks it used.</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1561,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Application running; a valid staff account exists.</t>
+          <t>Usher is logged in; the ticket exists.</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1573,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Staff authenticated with role-based access.</t>
+          <t>Ticket marked Used; entry granted or refused.</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1585,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>1. Enter username and password. 2. System validates and reads the role. 3. On success, the menu opens (full for Manager, selling for Cashier).</t>
+          <t>1. Scan/enter the ticket code. 2. Find ticket and showtime. 3. Check valid, right showtime, not used. 4. Mark Used and show 'Access granted'.</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1597,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2a. Invalid credentials -&gt; show 'Invalid login credentials', stay on login screen.</t>
+          <t>3a. Already used / wrong showtime -&gt; 'Invalid ticket', refuse entry.</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1608,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UC-16  —  Schedule Showtime</t>
+          <t>UC-52  —  Generate Sales Report</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -1064,7 +1621,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>UC-16</t>
+          <t>UC-52</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1633,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Schedule Showtime</t>
+          <t>Generate Sales Report</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1657,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Schedules a movie in a hall at a given date, time and ticket price.</t>
+          <t>Produces a report of tickets sold and revenue for a chosen period.</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1669,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Manager is logged in; at least one movie and one hall exist.</t>
+          <t>Manager is logged in.</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1681,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>A new showtime is stored.</t>
+          <t>A report is displayed/printed.</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1693,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>1. Open Showtime scheduling. 2. Choose movie and hall, enter date, time, ticket price. 3. Save. 4. Validate and store the showtime.</t>
+          <t>1. Choose the period (date range). 2. System totals tickets sold and revenue. 3. Display report with grand total.</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1705,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>3a. A showtime already exists for that hall at that date/time -&gt; clash error.</t>
+          <t>1a. No data in period -&gt; report shows zero totals.</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1716,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>UC-12  —  Add Movie</t>
+          <t>UC-01  —  Add Movie</t>
         </is>
       </c>
       <c r="B31" s="4" t="n"/>
@@ -1172,7 +1729,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>UC-12</t>
+          <t>UC-01</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1765,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Adds a new movie to the catalogue.</t>
+          <t>Adds a new movie to the catalogue (template for all Add/Update/Delete/Search use cases).</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1801,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>1. Open Movie Management. 2. Enter title, genre, duration, rating. 3. Save. 4. Validate and store.</t>
+          <t>1. Open the Movie form. 2. Enter title, genre, duration, language, rating. 3. Save. 4. Validate and store.</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1813,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>3a. Duplicate title / missing field -&gt; error, not saved.</t>
+          <t>3a. Duplicate / missing field -&gt; error, not saved.</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1828,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Replicate this template for: Update/Delete Movie, Manage Cinema Halls, Update/Delete Showtime, Set Ticket Pricing, Search Movies, View Showtimes, Cancel Ticket, Validate Ticket, View Sold Tickets, View Sales Report, Logout.</t>
+          <t>Replicate the CRUD template for every Add/Update/Delete/Search use case of Movie, Genre, Hall, Showtime, Customer, Staff, Booking, Ticket, Payment, Snack, Promotion. Write full specs for Post/Unpost Showtime, Select Seat, Apply Promotion, Add Payment, Generate Ticket, Issue Refund, the three reports, Manage User Roles, Login, Logout.</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1850,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1366,11 +1923,7 @@
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>UQ</t>
-        </is>
-      </c>
+      <c r="C5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1393,7 +1946,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>ENUM('MANAGER','CASHIER')</t>
+          <t>ENUM('MANAGER','CASHIER','USHER')</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr"/>
@@ -1465,64 +2018,64 @@
       </c>
       <c r="C13" s="9" t="inlineStr"/>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>movie</t>
-        </is>
-      </c>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>genre</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Key</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>movie_id</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>genre_id</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(120)</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr"/>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>genre</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -1532,82 +2085,86 @@
       </c>
       <c r="C19" s="9" t="inlineStr"/>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>duration</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>rating</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>VARCHAR(10)</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr"/>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>movie</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>cinema_hall</t>
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>movie_id</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(120)</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>hall_id</t>
+          <t>genre_id</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>FK -&gt; genre</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>hall_name</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(60)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr"/>
@@ -1615,100 +2172,92 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>capacity</t>
+          <t>language</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(40)</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr"/>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>showtime</t>
-        </is>
-      </c>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>cinema_hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Key</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>show_id</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>INT (auto)</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>movie_id</t>
+          <t>hall_id</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>INT (auto)</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>FK -&gt; movie</t>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>hall_id</t>
+          <t>hall_name</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; cinema_hall</t>
-        </is>
-      </c>
+          <t>VARCHAR(60)</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>show_date</t>
+          <t>hall_type</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr"/>
@@ -1716,78 +2265,78 @@
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>show_time</t>
+          <t>capacity</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>UQ(hall,date,time)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>ticket_price</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>DECIMAL(8,2)</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr"/>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>showtime</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>ticket</t>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Key</t>
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>ticket_id</t>
+          <t>movie_id</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>FK -&gt; movie</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>show_id</t>
+          <t>hall_id</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -1797,53 +2346,45 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>FK -&gt; showtime</t>
+          <t>FK -&gt; cinema_hall</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>customer_id</t>
+          <t>show_date</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>FK -&gt; customer</t>
-        </is>
-      </c>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>seat_number</t>
+          <t>show_time</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(8)</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>UQ(show,seat)</t>
-        </is>
-      </c>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>ticket_type</t>
+          <t>ticket_price</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>ENUM('Adult','Kid')</t>
+          <t>DECIMAL(8,2)</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr"/>
@@ -1851,37 +2392,655 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Posted','Unposted')</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>show_id</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; showtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>promotion_id</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; promotion (null)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>booking_datetime</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>DATETIME</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Confirmed','Cancelled')</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>total_amount</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>ticket_id</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>seat_number</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(8)</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
           <t>price</t>
         </is>
       </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B62" s="9" t="inlineStr">
         <is>
           <t>DECIMAL(8,2)</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>purchase_datetime</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Valid','Used','Refunded')</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>payment</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>payment_id</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Card','Mobile','Cash')</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
+          <t>payment_datetime</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="inlineStr">
         <is>
           <t>DATETIME</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr"/>
+      <c r="C71" s="9" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
+        <is>
+          <t>ENUM('Paid','Refunded')</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>snack</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>snack_id</t>
+        </is>
+      </c>
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(50)</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(30)</t>
+        </is>
+      </c>
+      <c r="C78" s="9" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>snack_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="9" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="9" t="inlineStr">
+        <is>
+          <t>snack_id</t>
+        </is>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C85" s="9" t="inlineStr">
+        <is>
+          <t>FK -&gt; snack</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>line_total</t>
+        </is>
+      </c>
+      <c r="B87" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(8,2)</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>promotion</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="9" t="inlineStr">
+        <is>
+          <t>promotion_id</t>
+        </is>
+      </c>
+      <c r="B91" s="9" t="inlineStr">
+        <is>
+          <t>INT (auto)</t>
+        </is>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B92" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="9" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B93" s="9" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="C93" s="9" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>discount_percent</t>
+        </is>
+      </c>
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>DECIMAL(5,2)</t>
+        </is>
+      </c>
+      <c r="C94" s="9" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="B95" s="9" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="C95" s="9" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="12">
+    <mergeCell ref="A47:C47"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A89:C89"/>
+    <mergeCell ref="A74:C74"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A81:C81"/>
+    <mergeCell ref="A65:C65"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove Usher actor; assign ticket validation to Cashier (3 clean actors)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Cashier, Usher</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Usher</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Manager, Cashier, Usher</t>
+          <t>Manager, Cashier</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Manager, Cashier, Usher</t>
+          <t>Manager, Cashier</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Usher</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Usher is logged in; the ticket exists.</t>
+          <t>Cashier is logged in; the ticket exists.</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>1. Scan/enter the ticket code. 2. Find ticket and showtime. 3. Check valid, right showtime, not used. 4. Mark Used and show 'Access granted'.</t>
+          <t>1. Scan/enter the ticket code. 2. Find ticket and showtime. 3. Check valid, right showtime, not used. 4. Mark Used and show 'Access granted' with the seat number.</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>ENUM('MANAGER','CASHIER','USHER')</t>
+          <t>ENUM('MANAGER','CASHIER')</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Clean actors (one primary per use case), keep 2 reports, 56 use cases
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Manager, Cashier</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Manager, Cashier</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Cashier, Customer (secondary)</t>
+          <t>Cashier (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Cashier, Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Cashier, Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Cashier, Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Cashier, Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Cashier, Customer (secondary)</t>
+          <t>Cashier (primary), Customer (secondary)</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Cashier, Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Generate Daily Revenue Report</t>
+          <t>Manage User Roles</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -1329,12 +1329,12 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Manage User Roles</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1344,27 +1344,12 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logout</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Manager, Cashier</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="n">
-        <v>57</v>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>Logout</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>Manager, Cashier</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1813,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Replicate the CRUD template for every Add/Update/Delete/Search use case of Movie, Genre, Hall, Showtime, Customer, Staff, Booking, Ticket, Payment, Snack, Promotion. Write full specs for Post/Unpost Showtime, Select Seat, Apply Promotion, Add Payment, Generate Ticket, Issue Refund, the three reports, Manage User Roles, Login, Logout.</t>
+          <t>Replicate the CRUD template for every Add/Update/Delete/Search use case of Movie, Genre, Hall, Showtime, Customer, Staff, Booking, Ticket, Payment, Snack, Promotion. Write full specs for Post/Unpost Showtime, Select Seat, Apply Promotion, Add Payment, Generate Ticket, Issue Refund, the two reports, Manage User Roles, Login, Logout.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Assign all Customer and Payment ops to Cashier (cleaner role split)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -794,7 +794,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Customer is a data entity, not an actor (counter-based system, mirrors example)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Cashier (primary), Customer (secondary)</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Cashier (primary), Customer (secondary)</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Creates a booking for a showtime: selects seats, applies any promotion, takes payment and issues the ticket.</t>
+          <t>The cashier creates a booking for a showtime on behalf of a customer: selects seats, applies any promotion, takes payment and issues the ticket.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add realistic Sell Snack use case; fix actor count to 2; renumber
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1119,12 +1119,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Add Promotion</t>
+          <t>Sell Snack</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Update Promotion</t>
+          <t>Add Promotion</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Delete Promotion</t>
+          <t>Update Promotion</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -1164,12 +1164,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Search Promotion by Code, Period</t>
+          <t>Delete Promotion</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -1179,12 +1179,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Post Showtime</t>
+          <t>Search Promotion by Code, Period</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Unpost Showtime</t>
+          <t>Post Showtime</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1209,12 +1209,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Select Seat</t>
+          <t>Unpost Showtime</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Apply Promotion to Booking</t>
+          <t>Select Seat</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Generate Ticket</t>
+          <t>Apply Promotion to Booking</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Validate Ticket at Entrance</t>
+          <t>Generate Ticket</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Issue Refund</t>
+          <t>Validate Ticket at Entrance</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Generate Sales Report</t>
+          <t>Issue Refund</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Cashier</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Generate Hall Occupancy Report</t>
+          <t>Generate Sales Report</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Manage User Roles</t>
+          <t>Generate Hall Occupancy Report</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -1329,12 +1329,12 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Manage User Roles</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Manager</t>
         </is>
       </c>
     </row>
@@ -1344,10 +1344,25 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Cashier</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
           <t>Logout</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -1485,7 +1500,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>UC-50  —  Validate Ticket at Entrance</t>
+          <t>UC-51  —  Validate Ticket at Entrance</t>
         </is>
       </c>
       <c r="B11" s="4" t="n"/>
@@ -1498,7 +1513,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>UC-50</t>
+          <t>UC-51</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1608,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UC-52  —  Generate Sales Report</t>
+          <t>UC-53  —  Generate Sales Report</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -1606,7 +1621,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>UC-52</t>
+          <t>UC-53</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1828,7 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Replicate the CRUD template for every Add/Update/Delete/Search use case of Movie, Genre, Hall, Showtime, Customer, Staff, Booking, Ticket, Payment, Snack, Promotion. Write full specs for Post/Unpost Showtime, Select Seat, Apply Promotion, Add Payment, Generate Ticket, Issue Refund, the two reports, Manage User Roles, Login, Logout.</t>
+          <t>Replicate the CRUD template for every Add/Update/Delete/Search use case of Movie, Genre, Hall, Showtime, Customer, Staff, Booking, Ticket, Payment, Snack, Promotion. Write full specs for Post/Unpost Showtime, Select Seat, Apply Promotion, Add Payment, Generate Ticket, Sell Snack, Issue Refund, the two reports, Manage User Roles, Login, Logout.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify PK data type to INT (drop auto)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -7421,7 +7421,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -7838,7 +7838,7 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
@@ -8193,7 +8193,7 @@
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
@@ -8303,7 +8303,7 @@
       </c>
       <c r="B76" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C76" s="9" t="inlineStr">
@@ -8383,7 +8383,7 @@
       </c>
       <c r="B83" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="B91" s="9" t="inlineStr">
         <is>
-          <t>INT (auto)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="C91" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Replace ENUM with VARCHAR(10) + value notes for simplicity
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -7477,10 +7477,14 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>ENUM('MANAGER','CASHIER')</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr"/>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Manager / Cashier</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -7928,10 +7932,14 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>ENUM('Posted','Unposted')</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr"/>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Posted / Unposted</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -8046,10 +8054,14 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>ENUM('Confirmed','Cancelled')</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr"/>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Confirmed / Cancelled</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
@@ -8156,10 +8168,14 @@
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>ENUM('Valid','Used','Refunded')</t>
-        </is>
-      </c>
-      <c r="C63" s="9" t="inlineStr"/>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>Valid / Used / Refunded</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -8240,10 +8256,14 @@
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>ENUM('Card','Mobile','Cash')</t>
-        </is>
-      </c>
-      <c r="C70" s="9" t="inlineStr"/>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>Card / Mobile / Cash</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
@@ -8266,10 +8286,14 @@
       </c>
       <c r="B72" s="9" t="inlineStr">
         <is>
-          <t>ENUM('Paid','Refunded')</t>
-        </is>
-      </c>
-      <c r="C72" s="9" t="inlineStr"/>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>Paid / Refunded</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Make use case specification tables plain black & white
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gShTjrczYVq9PahH9u6Mo
</commit_message>
<xml_diff>
--- a/cinema-management-system-analysis/Cinema_Management_System.xlsx
+++ b/cinema-management-system-analysis/Cinema_Management_System.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,10 @@
     <font>
       <i val="1"/>
       <color rgb="00595959"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
     </font>
     <font>
       <b val="1"/>
@@ -67,7 +71,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -89,11 +93,25 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -107,15 +125,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1411,7 +1432,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>UC-01</t>
         </is>
@@ -1423,7 +1444,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Add Movie</t>
         </is>
@@ -1435,7 +1456,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -1447,7 +1468,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Adds a new movie to the system.</t>
         </is>
@@ -1459,7 +1480,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>The Manager is logged in.</t>
         </is>
@@ -1471,7 +1492,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>A new movie record is stored.</t>
         </is>
@@ -1483,7 +1504,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>1. Open the Movie form. 2. Enter the movie details. 3. Click Save. 4. The system validates the data and stores the new movie.</t>
         </is>
@@ -1495,7 +1516,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>3a. A required field is missing or a duplicate exists → the system shows an error and nothing is saved.</t>
         </is>
@@ -1515,7 +1536,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>UC-02</t>
         </is>
@@ -1527,7 +1548,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Update Movie</t>
         </is>
@@ -1539,7 +1560,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -1551,7 +1572,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Modifies the details of an existing movie.</t>
         </is>
@@ -1563,7 +1584,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>The Manager is logged in.</t>
         </is>
@@ -1575,7 +1596,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>The movie record is updated.</t>
         </is>
@@ -1587,7 +1608,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>1. Search and select the movie. 2. Edit the details. 3. Click Save. 4. The system validates and updates the record.</t>
         </is>
@@ -1599,7 +1620,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>3a. Invalid data → error, no change is saved.</t>
         </is>
@@ -1619,7 +1640,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>UC-03</t>
         </is>
@@ -1631,7 +1652,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Delete Movie</t>
         </is>
@@ -1643,7 +1664,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -1655,7 +1676,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Removes a movie from the system.</t>
         </is>
@@ -1667,7 +1688,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>The Manager is logged in.</t>
         </is>
@@ -1679,7 +1700,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>The movie record is deleted.</t>
         </is>
@@ -1691,7 +1712,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>1. Select the movie. 2. Confirm the deletion. 3. The system removes the record.</t>
         </is>
@@ -1703,7 +1724,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>2a. The movie is referenced elsewhere → the deletion is blocked with a warning.</t>
         </is>
@@ -1723,7 +1744,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>UC-04</t>
         </is>
@@ -1735,7 +1756,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Search Movie by Title, Genre, Language</t>
         </is>
@@ -1747,7 +1768,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -1759,7 +1780,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>Finds movie records by title, genre, language.</t>
         </is>
@@ -1771,7 +1792,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>The Cashier is logged in.</t>
         </is>
@@ -1783,7 +1804,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>The matching records are displayed.</t>
         </is>
@@ -1795,7 +1816,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>1. Enter the search criteria (Title, Genre, Language). 2. The system displays the matching movie records.</t>
         </is>
@@ -1807,7 +1828,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>2a. No match → the system shows an empty result.</t>
         </is>
@@ -1827,7 +1848,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>UC-25</t>
         </is>
@@ -1839,7 +1860,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>Add Booking</t>
         </is>
@@ -1851,7 +1872,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -1863,7 +1884,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
         <is>
           <t>The cashier creates a booking for a showtime on behalf of a customer: selects seats, applies any promotion, takes payment and issues the ticket.</t>
         </is>
@@ -1875,7 +1896,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>The cashier is logged in; a posted showtime with a free seat exists.</t>
         </is>
@@ -1887,7 +1908,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t>A booking, ticket and payment are saved; the seats are marked sold.</t>
         </is>
@@ -1899,7 +1920,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>1. Select a posted showtime. 2. Select one or more seats («include» Select Seat). 3. Enter/select the customer. 4. (optional) Apply a promotion («extend» Apply Promotion). 5. Take payment («include» Add Payment). 6. Save the booking and issue the ticket («include» Generate Ticket); mark the seats sold. 7. Print/show the ticket.</t>
         </is>
@@ -1911,7 +1932,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B51" s="8" t="inlineStr">
         <is>
           <t>2a. Seat already sold → choose another seat. 5a. Payment fails → release the seats, no ticket.</t>
         </is>
@@ -1931,7 +1952,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>UC-48</t>
         </is>
@@ -1943,7 +1964,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B55" s="8" t="inlineStr">
         <is>
           <t>Select Seat</t>
         </is>
@@ -1955,7 +1976,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -1967,7 +1988,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="8" t="inlineStr">
         <is>
           <t>Chooses one or more available seats for a showtime.</t>
         </is>
@@ -1979,7 +2000,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>A showtime is selected; a seat map is displayed.</t>
         </is>
@@ -1991,7 +2012,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="8" t="inlineStr">
         <is>
           <t>The chosen seats are reserved for the booking.</t>
         </is>
@@ -2003,7 +2024,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>1. The system shows available seats. 2. The cashier selects the seat(s). 3. The seats are held.</t>
         </is>
@@ -2015,7 +2036,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B61" s="8" t="inlineStr">
         <is>
           <t>2a. Seat just taken → ask for another seat.</t>
         </is>
@@ -2035,7 +2056,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>UC-33</t>
         </is>
@@ -2047,7 +2068,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" s="8" t="inlineStr">
         <is>
           <t>Add Payment</t>
         </is>
@@ -2059,7 +2080,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -2071,7 +2092,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="8" t="inlineStr">
         <is>
           <t>Charges the customer for a booking.</t>
         </is>
@@ -2083,7 +2104,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>A booking with a total amount is awaiting payment.</t>
         </is>
@@ -2095,7 +2116,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B69" s="8" t="inlineStr">
         <is>
           <t>A payment record is created (Paid or Failed).</t>
         </is>
@@ -2107,7 +2128,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>1. Show the amount due and methods (Card, Mobile, Cash). 2. Choose a method. 3. Process payment, record as Paid.</t>
         </is>
@@ -2119,7 +2140,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B71" s="8" t="inlineStr">
         <is>
           <t>3a. Declined → record Failed; booking stays unpaid.</t>
         </is>
@@ -2139,7 +2160,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
         <is>
           <t>UC-50</t>
         </is>
@@ -2151,7 +2172,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B75" s="8" t="inlineStr">
         <is>
           <t>Generate Ticket</t>
         </is>
@@ -2163,7 +2184,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B76" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -2175,7 +2196,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B77" s="8" t="inlineStr">
         <is>
           <t>Issues the ticket(s) for a paid booking with a unique code.</t>
         </is>
@@ -2187,7 +2208,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B78" s="8" t="inlineStr">
         <is>
           <t>The booking is paid.</t>
         </is>
@@ -2199,7 +2220,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B79" s="8" t="inlineStr">
         <is>
           <t>Ticket(s) are created with status Valid and printed/shown.</t>
         </is>
@@ -2211,7 +2232,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B80" s="8" t="inlineStr">
         <is>
           <t>1. Create a ticket per seat with a unique code. 2. Print/show the ticket(s).</t>
         </is>
@@ -2223,7 +2244,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B81" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2243,7 +2264,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B84" s="8" t="inlineStr">
         <is>
           <t>UC-49</t>
         </is>
@@ -2255,7 +2276,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B85" s="8" t="inlineStr">
         <is>
           <t>Apply Promotion to Booking</t>
         </is>
@@ -2267,7 +2288,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B86" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -2279,7 +2300,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B87" s="3" t="inlineStr">
+      <c r="B87" s="8" t="inlineStr">
         <is>
           <t>Applies a valid promotion code to a booking to reduce the total.</t>
         </is>
@@ -2291,7 +2312,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B88" s="8" t="inlineStr">
         <is>
           <t>A booking is in progress; a valid promotion exists.</t>
         </is>
@@ -2303,7 +2324,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B89" s="3" t="inlineStr">
+      <c r="B89" s="8" t="inlineStr">
         <is>
           <t>The discount is applied and the total recalculated.</t>
         </is>
@@ -2315,7 +2336,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="B90" s="8" t="inlineStr">
         <is>
           <t>1. Enter the promotion code. 2. The system checks it is valid and in date. 3. Apply the discount.</t>
         </is>
@@ -2327,7 +2348,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B91" s="3" t="inlineStr">
+      <c r="B91" s="8" t="inlineStr">
         <is>
           <t>2a. Invalid/expired code → no discount; show a message.</t>
         </is>
@@ -2347,7 +2368,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B94" s="3" t="inlineStr">
+      <c r="B94" s="8" t="inlineStr">
         <is>
           <t>UC-52</t>
         </is>
@@ -2359,7 +2380,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B95" s="3" t="inlineStr">
+      <c r="B95" s="8" t="inlineStr">
         <is>
           <t>Issue Refund</t>
         </is>
@@ -2371,7 +2392,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B96" s="3" t="inlineStr">
+      <c r="B96" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -2383,7 +2404,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B97" s="3" t="inlineStr">
+      <c r="B97" s="8" t="inlineStr">
         <is>
           <t>Refunds a cancelled booking.</t>
         </is>
@@ -2395,7 +2416,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="B98" s="8" t="inlineStr">
         <is>
           <t>The booking is paid and being cancelled.</t>
         </is>
@@ -2407,7 +2428,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B99" s="8" t="inlineStr">
         <is>
           <t>A refund payment is recorded; the ticket status becomes Refunded.</t>
         </is>
@@ -2419,7 +2440,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B100" s="3" t="inlineStr">
+      <c r="B100" s="8" t="inlineStr">
         <is>
           <t>1. Select the cancelled booking. 2. Confirm the refund. 3. Record the refund and mark the ticket Refunded.</t>
         </is>
@@ -2431,7 +2452,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B101" s="3" t="inlineStr">
+      <c r="B101" s="8" t="inlineStr">
         <is>
           <t>2a. Booking not paid → nothing to refund.</t>
         </is>
@@ -2451,7 +2472,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B104" s="3" t="inlineStr">
+      <c r="B104" s="8" t="inlineStr">
         <is>
           <t>UC-51</t>
         </is>
@@ -2463,7 +2484,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B105" s="3" t="inlineStr">
+      <c r="B105" s="8" t="inlineStr">
         <is>
           <t>Validate Ticket at Entrance</t>
         </is>
@@ -2475,7 +2496,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B106" s="3" t="inlineStr">
+      <c r="B106" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -2487,7 +2508,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B107" s="3" t="inlineStr">
+      <c r="B107" s="8" t="inlineStr">
         <is>
           <t>Checks that a presented ticket is valid for the current showtime and marks it used.</t>
         </is>
@@ -2499,7 +2520,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B108" s="3" t="inlineStr">
+      <c r="B108" s="8" t="inlineStr">
         <is>
           <t>The cashier is logged in; the ticket exists.</t>
         </is>
@@ -2511,7 +2532,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B109" s="3" t="inlineStr">
+      <c r="B109" s="8" t="inlineStr">
         <is>
           <t>The ticket is marked Used; entry granted or refused.</t>
         </is>
@@ -2523,7 +2544,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B110" s="8" t="inlineStr">
         <is>
           <t>1. Scan/enter the ticket code. 2. Find the ticket and showtime. 3. Check it is Valid, for the right showtime and not used. 4. Mark Used and show 'Access granted' with the seat.</t>
         </is>
@@ -2535,7 +2556,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B111" s="8" t="inlineStr">
         <is>
           <t>3a. Already used / wrong showtime → 'Invalid ticket', refuse entry.</t>
         </is>
@@ -2555,7 +2576,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B114" s="3" t="inlineStr">
+      <c r="B114" s="8" t="inlineStr">
         <is>
           <t>UC-41</t>
         </is>
@@ -2567,7 +2588,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B115" s="3" t="inlineStr">
+      <c r="B115" s="8" t="inlineStr">
         <is>
           <t>Sell Snack</t>
         </is>
@@ -2579,7 +2600,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B116" s="3" t="inlineStr">
+      <c r="B116" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -2591,7 +2612,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B117" s="3" t="inlineStr">
+      <c r="B117" s="8" t="inlineStr">
         <is>
           <t>Sells one or more snacks to a customer and records the snack order.</t>
         </is>
@@ -2603,7 +2624,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B118" s="3" t="inlineStr">
+      <c r="B118" s="8" t="inlineStr">
         <is>
           <t>The cashier is logged in; snacks exist in the menu.</t>
         </is>
@@ -2615,7 +2636,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B119" s="3" t="inlineStr">
+      <c r="B119" s="8" t="inlineStr">
         <is>
           <t>A snack order is saved with its line(s) and total.</t>
         </is>
@@ -2627,7 +2648,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B120" s="3" t="inlineStr">
+      <c r="B120" s="8" t="inlineStr">
         <is>
           <t>1. Select the snack(s) and quantity. 2. The system computes the total. 3. Take payment. 4. Save the snack order.</t>
         </is>
@@ -2639,7 +2660,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B121" s="3" t="inlineStr">
+      <c r="B121" s="8" t="inlineStr">
         <is>
           <t>2a. Snack out of stock → choose another.</t>
         </is>
@@ -2659,7 +2680,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B124" s="3" t="inlineStr">
+      <c r="B124" s="8" t="inlineStr">
         <is>
           <t>UC-46</t>
         </is>
@@ -2671,7 +2692,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B125" s="3" t="inlineStr">
+      <c r="B125" s="8" t="inlineStr">
         <is>
           <t>Post Showtime</t>
         </is>
@@ -2683,7 +2704,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B126" s="3" t="inlineStr">
+      <c r="B126" s="8" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -2695,7 +2716,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B127" s="3" t="inlineStr">
+      <c r="B127" s="8" t="inlineStr">
         <is>
           <t>Publishes a showtime so it becomes available for selling tickets.</t>
         </is>
@@ -2707,7 +2728,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B128" s="3" t="inlineStr">
+      <c r="B128" s="8" t="inlineStr">
         <is>
           <t>The manager is logged in; the showtime exists.</t>
         </is>
@@ -2719,7 +2740,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B129" s="3" t="inlineStr">
+      <c r="B129" s="8" t="inlineStr">
         <is>
           <t>The showtime status becomes Posted.</t>
         </is>
@@ -2731,7 +2752,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B130" s="3" t="inlineStr">
+      <c r="B130" s="8" t="inlineStr">
         <is>
           <t>1. Select the showtime. 2. Click Post. 3. The status becomes Posted.</t>
         </is>
@@ -2743,7 +2764,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B131" s="3" t="inlineStr">
+      <c r="B131" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2763,7 +2784,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B134" s="3" t="inlineStr">
+      <c r="B134" s="8" t="inlineStr">
         <is>
           <t>UC-47</t>
         </is>
@@ -2775,7 +2796,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B135" s="3" t="inlineStr">
+      <c r="B135" s="8" t="inlineStr">
         <is>
           <t>Unpost Showtime</t>
         </is>
@@ -2787,7 +2808,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B136" s="3" t="inlineStr">
+      <c r="B136" s="8" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -2799,7 +2820,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B137" s="3" t="inlineStr">
+      <c r="B137" s="8" t="inlineStr">
         <is>
           <t>Hides a showtime so tickets can no longer be sold for it.</t>
         </is>
@@ -2811,7 +2832,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B138" s="3" t="inlineStr">
+      <c r="B138" s="8" t="inlineStr">
         <is>
           <t>The manager is logged in; the showtime is Posted.</t>
         </is>
@@ -2823,7 +2844,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B139" s="3" t="inlineStr">
+      <c r="B139" s="8" t="inlineStr">
         <is>
           <t>The showtime status becomes Unposted.</t>
         </is>
@@ -2835,7 +2856,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B140" s="3" t="inlineStr">
+      <c r="B140" s="8" t="inlineStr">
         <is>
           <t>1. Select the showtime. 2. Click Unpost. 3. The status becomes Unposted.</t>
         </is>
@@ -2847,7 +2868,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B141" s="3" t="inlineStr">
+      <c r="B141" s="8" t="inlineStr">
         <is>
           <t>2a. Tickets already sold → warn before unposting.</t>
         </is>
@@ -2867,7 +2888,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B144" s="3" t="inlineStr">
+      <c r="B144" s="8" t="inlineStr">
         <is>
           <t>UC-53</t>
         </is>
@@ -2879,7 +2900,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B145" s="8" t="inlineStr">
         <is>
           <t>Generate Sales Report</t>
         </is>
@@ -2891,7 +2912,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B146" s="3" t="inlineStr">
+      <c r="B146" s="8" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -2903,7 +2924,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B147" s="3" t="inlineStr">
+      <c r="B147" s="8" t="inlineStr">
         <is>
           <t>Produces a report of tickets sold and revenue for a chosen period.</t>
         </is>
@@ -2915,7 +2936,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B148" s="3" t="inlineStr">
+      <c r="B148" s="8" t="inlineStr">
         <is>
           <t>The manager is logged in.</t>
         </is>
@@ -2927,7 +2948,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B149" s="8" t="inlineStr">
         <is>
           <t>A report is displayed/printed.</t>
         </is>
@@ -2939,7 +2960,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B150" s="8" t="inlineStr">
         <is>
           <t>1. Choose the period. 2. The system totals tickets sold and revenue. 3. Display the report with a grand total.</t>
         </is>
@@ -2951,7 +2972,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B151" s="3" t="inlineStr">
+      <c r="B151" s="8" t="inlineStr">
         <is>
           <t>1a. No data → zero totals.</t>
         </is>
@@ -2971,7 +2992,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B154" s="3" t="inlineStr">
+      <c r="B154" s="8" t="inlineStr">
         <is>
           <t>UC-54</t>
         </is>
@@ -2983,7 +3004,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B155" s="3" t="inlineStr">
+      <c r="B155" s="8" t="inlineStr">
         <is>
           <t>Generate Hall Occupancy Report</t>
         </is>
@@ -2995,7 +3016,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B156" s="3" t="inlineStr">
+      <c r="B156" s="8" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -3007,7 +3028,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B157" s="3" t="inlineStr">
+      <c r="B157" s="8" t="inlineStr">
         <is>
           <t>Shows, per showtime, the seats sold versus capacity and the occupancy rate.</t>
         </is>
@@ -3019,7 +3040,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B158" s="3" t="inlineStr">
+      <c r="B158" s="8" t="inlineStr">
         <is>
           <t>The manager is logged in.</t>
         </is>
@@ -3031,7 +3052,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B159" s="3" t="inlineStr">
+      <c r="B159" s="8" t="inlineStr">
         <is>
           <t>An occupancy report is displayed/printed.</t>
         </is>
@@ -3043,7 +3064,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B160" s="3" t="inlineStr">
+      <c r="B160" s="8" t="inlineStr">
         <is>
           <t>1. Choose the period/hall. 2. The system computes seats sold / capacity per showtime. 3. Display the report.</t>
         </is>
@@ -3055,7 +3076,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B161" s="3" t="inlineStr">
+      <c r="B161" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3075,7 +3096,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B164" s="3" t="inlineStr">
+      <c r="B164" s="8" t="inlineStr">
         <is>
           <t>UC-55</t>
         </is>
@@ -3087,7 +3108,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B165" s="3" t="inlineStr">
+      <c r="B165" s="8" t="inlineStr">
         <is>
           <t>Manage User Roles</t>
         </is>
@@ -3099,7 +3120,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B166" s="3" t="inlineStr">
+      <c r="B166" s="8" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -3111,7 +3132,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B167" s="3" t="inlineStr">
+      <c r="B167" s="8" t="inlineStr">
         <is>
           <t>Assigns or changes the role (Manager/Cashier) of a staff account.</t>
         </is>
@@ -3123,7 +3144,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B168" s="3" t="inlineStr">
+      <c r="B168" s="8" t="inlineStr">
         <is>
           <t>The manager is logged in.</t>
         </is>
@@ -3135,7 +3156,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B169" s="3" t="inlineStr">
+      <c r="B169" s="8" t="inlineStr">
         <is>
           <t>The staff member's role is updated.</t>
         </is>
@@ -3147,7 +3168,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B170" s="3" t="inlineStr">
+      <c r="B170" s="8" t="inlineStr">
         <is>
           <t>1. Select the staff account. 2. Choose the role. 3. Save.</t>
         </is>
@@ -3159,7 +3180,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B171" s="3" t="inlineStr">
+      <c r="B171" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3179,7 +3200,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B174" s="3" t="inlineStr">
+      <c r="B174" s="8" t="inlineStr">
         <is>
           <t>UC-56</t>
         </is>
@@ -3191,7 +3212,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B175" s="3" t="inlineStr">
+      <c r="B175" s="8" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
@@ -3203,7 +3224,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B176" s="3" t="inlineStr">
+      <c r="B176" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -3215,7 +3236,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B177" s="3" t="inlineStr">
+      <c r="B177" s="8" t="inlineStr">
         <is>
           <t>Authenticates a staff member and opens the menu according to their role.</t>
         </is>
@@ -3227,7 +3248,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B178" s="3" t="inlineStr">
+      <c r="B178" s="8" t="inlineStr">
         <is>
           <t>The application is running; a valid staff account exists.</t>
         </is>
@@ -3239,7 +3260,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B179" s="3" t="inlineStr">
+      <c r="B179" s="8" t="inlineStr">
         <is>
           <t>The staff member is authenticated with role-based access.</t>
         </is>
@@ -3251,7 +3272,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B180" s="3" t="inlineStr">
+      <c r="B180" s="8" t="inlineStr">
         <is>
           <t>1. Enter username and password. 2. The system validates and reads the role. 3. Open the menu (full for Manager, selling for Cashier).</t>
         </is>
@@ -3263,7 +3284,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B181" s="3" t="inlineStr">
+      <c r="B181" s="8" t="inlineStr">
         <is>
           <t>2a. Invalid credentials → show 'Invalid login credentials', stay on the login screen.</t>
         </is>
@@ -3283,7 +3304,7 @@
           <t>Use Case ID</t>
         </is>
       </c>
-      <c r="B184" s="3" t="inlineStr">
+      <c r="B184" s="8" t="inlineStr">
         <is>
           <t>UC-57</t>
         </is>
@@ -3295,7 +3316,7 @@
           <t>Use Case Name</t>
         </is>
       </c>
-      <c r="B185" s="3" t="inlineStr">
+      <c r="B185" s="8" t="inlineStr">
         <is>
           <t>Logout</t>
         </is>
@@ -3307,7 +3328,7 @@
           <t>Actor(s)</t>
         </is>
       </c>
-      <c r="B186" s="3" t="inlineStr">
+      <c r="B186" s="8" t="inlineStr">
         <is>
           <t>Cashier</t>
         </is>
@@ -3319,7 +3340,7 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B187" s="3" t="inlineStr">
+      <c r="B187" s="8" t="inlineStr">
         <is>
           <t>Ends the staff member's session securely.</t>
         </is>
@@ -3331,7 +3352,7 @@
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="B188" s="3" t="inlineStr">
+      <c r="B188" s="8" t="inlineStr">
         <is>
           <t>A staff member is logged in.</t>
         </is>
@@ -3343,7 +3364,7 @@
           <t>Postconditions</t>
         </is>
       </c>
-      <c r="B189" s="3" t="inlineStr">
+      <c r="B189" s="8" t="inlineStr">
         <is>
           <t>The session is closed; the login screen is shown.</t>
         </is>
@@ -3355,7 +3376,7 @@
           <t>Main Flow</t>
         </is>
       </c>
-      <c r="B190" s="3" t="inlineStr">
+      <c r="B190" s="8" t="inlineStr">
         <is>
           <t>1. Click Logout. 2. The system closes the session and returns to the login screen.</t>
         </is>
@@ -3367,7 +3388,7 @@
           <t>Alternative Flows</t>
         </is>
       </c>
-      <c r="B191" s="3" t="inlineStr">
+      <c r="B191" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3415,1197 +3436,1197 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>staff</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>staff_id</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>full_name</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(100)</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr"/>
+      <c r="C4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>username</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr"/>
+      <c r="C5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(255)</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr"/>
+      <c r="C6" s="11" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(10)</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Manager / Cashier</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>customer</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>full_name</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(100)</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr"/>
+      <c r="C12" s="11" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(20)</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr"/>
+      <c r="C13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(100)</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr"/>
+      <c r="C14" s="11" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>genre</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>genre_id</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr"/>
+      <c r="C19" s="11" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>movie</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>movie_id</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(120)</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr"/>
+      <c r="C24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>genre_id</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; genre</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>duration</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr"/>
+      <c r="C26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>language</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(40)</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr"/>
+      <c r="C27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>rating</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(10)</t>
         </is>
       </c>
-      <c r="C28" s="10" t="inlineStr"/>
+      <c r="C28" s="11" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>cinema_hall</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>hall_id</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>hall_name</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(60)</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr"/>
+      <c r="C33" s="11" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>hall_type</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(20)</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr"/>
+      <c r="C34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>capacity</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr"/>
+      <c r="C35" s="11" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>showtime</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>show_id</t>
         </is>
       </c>
-      <c r="B39" s="10" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C39" s="10" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>movie_id</t>
         </is>
       </c>
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; movie</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>hall_id</t>
         </is>
       </c>
-      <c r="B41" s="10" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; cinema_hall</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="inlineStr">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>show_date</t>
         </is>
       </c>
-      <c r="B42" s="10" t="inlineStr">
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
-      <c r="C42" s="10" t="inlineStr"/>
+      <c r="C42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="10" t="inlineStr">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>show_time</t>
         </is>
       </c>
-      <c r="B43" s="10" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>TIME</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr"/>
+      <c r="C43" s="11" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>ticket_price</t>
         </is>
       </c>
-      <c r="B44" s="10" t="inlineStr">
+      <c r="B44" s="11" t="inlineStr">
         <is>
           <t>DECIMAL(8,2)</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr"/>
+      <c r="C44" s="11" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="10" t="inlineStr">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(10)</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>Posted / Unposted</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>booking</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="inlineStr">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B48" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C48" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="inlineStr">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>booking_id</t>
         </is>
       </c>
-      <c r="B49" s="10" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
+      <c r="C49" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="A50" s="11" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="B50" s="10" t="inlineStr">
+      <c r="B50" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
+      <c r="C50" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; customer</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="10" t="inlineStr">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>show_id</t>
         </is>
       </c>
-      <c r="B51" s="10" t="inlineStr">
+      <c r="B51" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; showtime</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>promotion_id</t>
         </is>
       </c>
-      <c r="B52" s="10" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
+      <c r="C52" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; promotion (null)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="10" t="inlineStr">
+      <c r="A53" s="11" t="inlineStr">
         <is>
           <t>booking_datetime</t>
         </is>
       </c>
-      <c r="B53" s="10" t="inlineStr">
+      <c r="B53" s="11" t="inlineStr">
         <is>
           <t>DATETIME</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr"/>
+      <c r="C53" s="11" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B54" s="10" t="inlineStr">
+      <c r="B54" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(10)</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
+      <c r="C54" s="11" t="inlineStr">
         <is>
           <t>Confirmed / Cancelled</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="10" t="inlineStr">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>total_amount</t>
         </is>
       </c>
-      <c r="B55" s="10" t="inlineStr">
+      <c r="B55" s="11" t="inlineStr">
         <is>
           <t>DECIMAL(8,2)</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr"/>
+      <c r="C55" s="11" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="A57" s="9" t="inlineStr">
         <is>
           <t>ticket</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="9" t="inlineStr">
+      <c r="A58" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B58" s="9" t="inlineStr">
+      <c r="B58" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C58" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="10" t="inlineStr">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>ticket_id</t>
         </is>
       </c>
-      <c r="B59" s="10" t="inlineStr">
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="10" t="inlineStr">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>booking_id</t>
         </is>
       </c>
-      <c r="B60" s="10" t="inlineStr">
+      <c r="B60" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; booking</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="inlineStr">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t>seat_number</t>
         </is>
       </c>
-      <c r="B61" s="10" t="inlineStr">
+      <c r="B61" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(8)</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr"/>
+      <c r="C61" s="11" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="inlineStr">
+      <c r="A62" s="11" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="B62" s="10" t="inlineStr">
+      <c r="B62" s="11" t="inlineStr">
         <is>
           <t>DECIMAL(8,2)</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr"/>
+      <c r="C62" s="11" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B63" s="10" t="inlineStr">
+      <c r="B63" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(10)</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
+      <c r="C63" s="11" t="inlineStr">
         <is>
           <t>Valid / Used / Refunded</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="A65" s="9" t="inlineStr">
         <is>
           <t>payment</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="9" t="inlineStr">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B66" s="9" t="inlineStr">
+      <c r="B66" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C66" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="10" t="inlineStr">
+      <c r="A67" s="11" t="inlineStr">
         <is>
           <t>payment_id</t>
         </is>
       </c>
-      <c r="B67" s="10" t="inlineStr">
+      <c r="B67" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
+      <c r="C67" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="10" t="inlineStr">
+      <c r="A68" s="11" t="inlineStr">
         <is>
           <t>booking_id</t>
         </is>
       </c>
-      <c r="B68" s="10" t="inlineStr">
+      <c r="B68" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
+      <c r="C68" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; booking</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="10" t="inlineStr">
+      <c r="A69" s="11" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="B69" s="10" t="inlineStr">
+      <c r="B69" s="11" t="inlineStr">
         <is>
           <t>DECIMAL(8,2)</t>
         </is>
       </c>
-      <c r="C69" s="10" t="inlineStr"/>
+      <c r="C69" s="11" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="10" t="inlineStr">
+      <c r="A70" s="11" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="B70" s="10" t="inlineStr">
+      <c r="B70" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(10)</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
+      <c r="C70" s="11" t="inlineStr">
         <is>
           <t>Card / Mobile / Cash</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="10" t="inlineStr">
+      <c r="A71" s="11" t="inlineStr">
         <is>
           <t>payment_datetime</t>
         </is>
       </c>
-      <c r="B71" s="10" t="inlineStr">
+      <c r="B71" s="11" t="inlineStr">
         <is>
           <t>DATETIME</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr"/>
+      <c r="C71" s="11" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="10" t="inlineStr">
+      <c r="A72" s="11" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B72" s="10" t="inlineStr">
+      <c r="B72" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(10)</t>
         </is>
       </c>
-      <c r="C72" s="10" t="inlineStr">
+      <c r="C72" s="11" t="inlineStr">
         <is>
           <t>Paid / Refunded</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+      <c r="A74" s="9" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="9" t="inlineStr">
+      <c r="A75" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B75" s="9" t="inlineStr">
+      <c r="B75" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C75" s="9" t="inlineStr">
+      <c r="C75" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="10" t="inlineStr">
+      <c r="A76" s="11" t="inlineStr">
         <is>
           <t>snack_id</t>
         </is>
       </c>
-      <c r="B76" s="10" t="inlineStr">
+      <c r="B76" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C76" s="10" t="inlineStr">
+      <c r="C76" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="10" t="inlineStr">
+      <c r="A77" s="11" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B77" s="10" t="inlineStr">
+      <c r="B77" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(50)</t>
         </is>
       </c>
-      <c r="C77" s="10" t="inlineStr"/>
+      <c r="C77" s="11" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="10" t="inlineStr">
+      <c r="A78" s="11" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="B78" s="10" t="inlineStr">
+      <c r="B78" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(30)</t>
         </is>
       </c>
-      <c r="C78" s="10" t="inlineStr"/>
+      <c r="C78" s="11" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="10" t="inlineStr">
+      <c r="A79" s="11" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="B79" s="10" t="inlineStr">
+      <c r="B79" s="11" t="inlineStr">
         <is>
           <t>DECIMAL(8,2)</t>
         </is>
       </c>
-      <c r="C79" s="10" t="inlineStr"/>
+      <c r="C79" s="11" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="8" t="inlineStr">
+      <c r="A81" s="9" t="inlineStr">
         <is>
           <t>snack_order</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="9" t="inlineStr">
+      <c r="A82" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B82" s="9" t="inlineStr">
+      <c r="B82" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C82" s="9" t="inlineStr">
+      <c r="C82" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="10" t="inlineStr">
+      <c r="A83" s="11" t="inlineStr">
         <is>
           <t>order_id</t>
         </is>
       </c>
-      <c r="B83" s="10" t="inlineStr">
+      <c r="B83" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C83" s="10" t="inlineStr">
+      <c r="C83" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="10" t="inlineStr">
+      <c r="A84" s="11" t="inlineStr">
         <is>
           <t>booking_id</t>
         </is>
       </c>
-      <c r="B84" s="10" t="inlineStr">
+      <c r="B84" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C84" s="10" t="inlineStr">
+      <c r="C84" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; booking</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="10" t="inlineStr">
+      <c r="A85" s="11" t="inlineStr">
         <is>
           <t>snack_id</t>
         </is>
       </c>
-      <c r="B85" s="10" t="inlineStr">
+      <c r="B85" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C85" s="10" t="inlineStr">
+      <c r="C85" s="11" t="inlineStr">
         <is>
           <t>FK -&gt; snack</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="10" t="inlineStr">
+      <c r="A86" s="11" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="B86" s="10" t="inlineStr">
+      <c r="B86" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C86" s="10" t="inlineStr"/>
+      <c r="C86" s="11" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="10" t="inlineStr">
+      <c r="A87" s="11" t="inlineStr">
         <is>
           <t>line_total</t>
         </is>
       </c>
-      <c r="B87" s="10" t="inlineStr">
+      <c r="B87" s="11" t="inlineStr">
         <is>
           <t>DECIMAL(8,2)</t>
         </is>
       </c>
-      <c r="C87" s="10" t="inlineStr"/>
+      <c r="C87" s="11" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="inlineStr">
+      <c r="A89" s="9" t="inlineStr">
         <is>
           <t>promotion</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="9" t="inlineStr">
+      <c r="A90" s="10" t="inlineStr">
         <is>
           <t>Attribute</t>
         </is>
       </c>
-      <c r="B90" s="9" t="inlineStr">
+      <c r="B90" s="10" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="C90" s="9" t="inlineStr">
+      <c r="C90" s="10" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="10" t="inlineStr">
+      <c r="A91" s="11" t="inlineStr">
         <is>
           <t>promotion_id</t>
         </is>
       </c>
-      <c r="B91" s="10" t="inlineStr">
+      <c r="B91" s="11" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="C91" s="10" t="inlineStr">
+      <c r="C91" s="11" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="10" t="inlineStr">
+      <c r="A92" s="11" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B92" s="10" t="inlineStr">
+      <c r="B92" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(20)</t>
         </is>
       </c>
-      <c r="C92" s="10" t="inlineStr"/>
+      <c r="C92" s="11" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="10" t="inlineStr">
+      <c r="A93" s="11" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B93" s="10" t="inlineStr">
+      <c r="B93" s="11" t="inlineStr">
         <is>
           <t>VARCHAR(100)</t>
         </is>
       </c>
-      <c r="C93" s="10" t="inlineStr"/>
+      <c r="C93" s="11" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="10" t="inlineStr">
+      <c r="A94" s="11" t="inlineStr">
         <is>
           <t>discount_percent</t>
         </is>
       </c>
-      <c r="B94" s="10" t="inlineStr">
+      <c r="B94" s="11" t="inlineStr">
         <is>
           <t>DECIMAL(5,2)</t>
         </is>
       </c>
-      <c r="C94" s="10" t="inlineStr"/>
+      <c r="C94" s="11" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="10" t="inlineStr">
+      <c r="A95" s="11" t="inlineStr">
         <is>
           <t>start_date</t>
         </is>
       </c>
-      <c r="B95" s="10" t="inlineStr">
+      <c r="B95" s="11" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
-      <c r="C95" s="10" t="inlineStr"/>
+      <c r="C95" s="11" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="10" t="inlineStr">
+      <c r="A96" s="11" t="inlineStr">
         <is>
           <t>end_date</t>
         </is>
       </c>
-      <c r="B96" s="10" t="inlineStr">
+      <c r="B96" s="11" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
-      <c r="C96" s="10" t="inlineStr"/>
+      <c r="C96" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>